<commit_message>
chore(auto): updated m3u8 links & playlist 6
</commit_message>
<xml_diff>
--- a/updated_videos_with_links.xlsx
+++ b/updated_videos_with_links.xlsx
@@ -472,7 +472,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://play.zephyrflick.top/cdn/hls/43152b16552a7b2461820cf065a4d042/master.m3u8?md5=I_Y9uFK6jPEJGgMFq_Rp7A&amp;expires=1769280732</t>
+          <t>https://play.zephyrflick.top/cdn/hls/43152b16552a7b2461820cf065a4d042/master.m3u8?md5=Eg6HYnG_3kzr3YKl7idXuA&amp;expires=1769281970</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://play.zephyrflick.top/cdn/hls/41900a626604bd5c1ff20add3ca2712a/master.m3u8?md5=i2mrICjHjR1HSawHLrUxyQ&amp;expires=1769280752</t>
+          <t>https://play.zephyrflick.top/cdn/hls/41900a626604bd5c1ff20add3ca2712a/master.m3u8?md5=RkujlnrOPdria7ltcd-8kA&amp;expires=1769281990</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://play.zephyrflick.top/cdn/hls/e3d1480b3031f637bba3412a2371f5ee/master.m3u8?md5=ZXNMBybYC4BpkV2hZTQ3Jw&amp;expires=1769280769</t>
+          <t>https://prd.jwpltx.com/v1/jwplayer6/ping.gif?h=936236969&amp;e=e&amp;n=4745213810198310&amp;aid=I9GYCF3cEeOTIBIxOQfUww&amp;amp=0&amp;at=1&amp;c=-1&amp;ccp=0&amp;cp=0&amp;d=1&amp;eb=1&amp;ed=2&amp;emi=1uiexz3citi3&amp;i=1&amp;lid=qexxzk4kwpah&amp;lsa=read&amp;mt=0&amp;pbd=1&amp;pbr=1&amp;pgi=azpnve1cdjau&amp;ph=0&amp;pii=0&amp;pl=0&amp;plc=1&amp;pli=g7cofhyn2v88&amp;pp=hlsjs&amp;prc=1&amp;ps=0&amp;pss=1&amp;pt=watchanimeworld.net&amp;pu=https%3A%2F%2Fwatchanimeworld.net%2F&amp;pv=8.33.1&amp;pyc=0&amp;s=0&amp;sdk=0&amp;ss=1&amp;stc=1&amp;stpe=0&amp;t=Shinchan%20-%20Season%2015%20-%20Episode%2003&amp;tv=4.0.3&amp;vb=0&amp;vi=0&amp;vl=90&amp;wd=0&amp;ab=1&amp;cae=0&amp;cb=0&amp;cdid=player&amp;cme=0&amp;dd=1&amp;flc=0&amp;fv=&amp;ga=0&amp;lng=en&amp;mk=hls&amp;mu=https%3A%2F%2Fplay.zephyrflick.top%2Fcdn%2Fhls%2Fe3d1480b3031f637bba3412a2371f5ee%2Fmaster.m3u8%3Fmd5%3DPudj7i5dF3uKLOfGjsyMNQ%26expires%3D1769282011&amp;pbc=1&amp;pd=3&amp;plng=en&amp;plt=600&amp;pni=1&amp;po=1&amp;sn=%7B%22name%22%3A%22alaska%22%7D&amp;sp=0&amp;st=120&amp;sa=1769274812196</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://play.zephyrflick.top/cdn/hls/98ef76b70cf62a93cc9753d70c010c25/master.m3u8?md5=V18IeEeNc8TMTP8cwisFTQ&amp;expires=1769280788</t>
+          <t>https://play.zephyrflick.top/cdn/hls/98ef76b70cf62a93cc9753d70c010c25/master.m3u8?md5=PKvadQxi3QJW56NR9gG9Iw&amp;expires=1769282031</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://play.zephyrflick.top/cdn/hls/6adbd64bdd5d9b3772de92566dc6dbc3/master.m3u8?md5=4fsitM2npNsGTdJ8irVTFA&amp;expires=1769280806</t>
+          <t>https://play.zephyrflick.top/cdn/hls/6adbd64bdd5d9b3772de92566dc6dbc3/master.m3u8?md5=mMW7k-9Zcy_Yq3jW-vL4wA&amp;expires=1769282049</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://play.zephyrflick.top/cdn/hls/35aa6d133de948464406d6b4b1a36a5b/master.m3u8?md5=oLECwL7jzUt86dckfUZCJQ&amp;expires=1769280823</t>
+          <t>https://play.zephyrflick.top/cdn/hls/35aa6d133de948464406d6b4b1a36a5b/master.m3u8?md5=iboTh7Z2ebKuuLV6gJA9zw&amp;expires=1769282067</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://play.zephyrflick.top/cdn/hls/74a143b078d25bb8af25b4260363c1ab/master.m3u8?md5=cUASvH5ZcY8dSJGsYtvJKQ&amp;expires=1769280842</t>
+          <t>https://play.zephyrflick.top/cdn/hls/74a143b078d25bb8af25b4260363c1ab/master.m3u8?md5=OQ6g27JJV8Bylw0MNGv0vQ&amp;expires=1769282087</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(auto): updated m3u8 links & playlist 7
</commit_message>
<xml_diff>
--- a/updated_videos_with_links.xlsx
+++ b/updated_videos_with_links.xlsx
@@ -472,7 +472,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://play.zephyrflick.top/cdn/hls/43152b16552a7b2461820cf065a4d042/master.m3u8?md5=Eg6HYnG_3kzr3YKl7idXuA&amp;expires=1769281970</t>
+          <t>https://play.zephyrflick.top/cdn/hls/43152b16552a7b2461820cf065a4d042/master.m3u8?md5=VKgPj2bExNQEYvypkh21nw&amp;expires=1769283308</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://play.zephyrflick.top/cdn/hls/41900a626604bd5c1ff20add3ca2712a/master.m3u8?md5=RkujlnrOPdria7ltcd-8kA&amp;expires=1769281990</t>
+          <t>https://play.zephyrflick.top/cdn/hls/41900a626604bd5c1ff20add3ca2712a/master.m3u8?md5=XCOozenLJK8iI2s1kvnIjQ&amp;expires=1769283341</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://prd.jwpltx.com/v1/jwplayer6/ping.gif?h=936236969&amp;e=e&amp;n=4745213810198310&amp;aid=I9GYCF3cEeOTIBIxOQfUww&amp;amp=0&amp;at=1&amp;c=-1&amp;ccp=0&amp;cp=0&amp;d=1&amp;eb=1&amp;ed=2&amp;emi=1uiexz3citi3&amp;i=1&amp;lid=qexxzk4kwpah&amp;lsa=read&amp;mt=0&amp;pbd=1&amp;pbr=1&amp;pgi=azpnve1cdjau&amp;ph=0&amp;pii=0&amp;pl=0&amp;plc=1&amp;pli=g7cofhyn2v88&amp;pp=hlsjs&amp;prc=1&amp;ps=0&amp;pss=1&amp;pt=watchanimeworld.net&amp;pu=https%3A%2F%2Fwatchanimeworld.net%2F&amp;pv=8.33.1&amp;pyc=0&amp;s=0&amp;sdk=0&amp;ss=1&amp;stc=1&amp;stpe=0&amp;t=Shinchan%20-%20Season%2015%20-%20Episode%2003&amp;tv=4.0.3&amp;vb=0&amp;vi=0&amp;vl=90&amp;wd=0&amp;ab=1&amp;cae=0&amp;cb=0&amp;cdid=player&amp;cme=0&amp;dd=1&amp;flc=0&amp;fv=&amp;ga=0&amp;lng=en&amp;mk=hls&amp;mu=https%3A%2F%2Fplay.zephyrflick.top%2Fcdn%2Fhls%2Fe3d1480b3031f637bba3412a2371f5ee%2Fmaster.m3u8%3Fmd5%3DPudj7i5dF3uKLOfGjsyMNQ%26expires%3D1769282011&amp;pbc=1&amp;pd=3&amp;plng=en&amp;plt=600&amp;pni=1&amp;po=1&amp;sn=%7B%22name%22%3A%22alaska%22%7D&amp;sp=0&amp;st=120&amp;sa=1769274812196</t>
+          <t>https://play.zephyrflick.top/cdn/hls/e3d1480b3031f637bba3412a2371f5ee/master.m3u8?md5=_3IB4s0GwvHS6GmlQvqa3A&amp;expires=1769283376</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://play.zephyrflick.top/cdn/hls/98ef76b70cf62a93cc9753d70c010c25/master.m3u8?md5=PKvadQxi3QJW56NR9gG9Iw&amp;expires=1769282031</t>
+          <t>https://play.zephyrflick.top/cdn/hls/98ef76b70cf62a93cc9753d70c010c25/master.m3u8?md5=GGw-qkGJJ6WeWI9uFdtsYg&amp;expires=1769283409</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://play.zephyrflick.top/cdn/hls/6adbd64bdd5d9b3772de92566dc6dbc3/master.m3u8?md5=mMW7k-9Zcy_Yq3jW-vL4wA&amp;expires=1769282049</t>
+          <t>https://play.zephyrflick.top/cdn/hls/6adbd64bdd5d9b3772de92566dc6dbc3/master.m3u8?md5=kXvIUO-pSojZ-IqoTLFI_Q&amp;expires=1769283446</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://play.zephyrflick.top/cdn/hls/35aa6d133de948464406d6b4b1a36a5b/master.m3u8?md5=iboTh7Z2ebKuuLV6gJA9zw&amp;expires=1769282067</t>
+          <t>https://play.zephyrflick.top/cdn/hls/35aa6d133de948464406d6b4b1a36a5b/master.m3u8?md5=lHs-sGivbULuz64_kOAWbg&amp;expires=1769283479</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://play.zephyrflick.top/cdn/hls/74a143b078d25bb8af25b4260363c1ab/master.m3u8?md5=OQ6g27JJV8Bylw0MNGv0vQ&amp;expires=1769282087</t>
+          <t>https://play.zephyrflick.top/cdn/hls/74a143b078d25bb8af25b4260363c1ab/master.m3u8?md5=llN8A0zEUzbgS0dq5GqpWw&amp;expires=1769283517</t>
         </is>
       </c>
     </row>

</xml_diff>